<commit_message>
Cargar clientes faltantes en permisos y aviso de cliente sin lista, estados de cuentas
</commit_message>
<xml_diff>
--- a/excel/GRUPOS_CLIENTES.xlsx
+++ b/excel/GRUPOS_CLIENTES.xlsx
@@ -54,56 +54,42 @@
     <t>RECURRENTE_&gt;_500K</t>
   </si>
   <si>
-    <t>936.940.973.992.997.10163.20113.20159.20166.20173.20180.20200.20258.20272.20275.20290.20291.20331.40137.40143.50444.50607.50622.50819.50821.50825.60165.60190.60195.60202.60205.60206.60215.61004.70102.70638.90668</t>
-  </si>
-  <si>
     <t>233.10167.20234.20292.20357.20379.20385.50102.50818.60124.60139.60158.60174.60258.70101.3.70114.20129</t>
   </si>
   <si>
     <t>949.1218.1959.5625.1817.5737</t>
   </si>
   <si>
-    <t>33.237.251.308.946.950.952.958.963.965.969.10165.20101.20110.20128.20148.20164.20236.20241.20246.20271.20284.20293.20309.20351.20380.20163.50815.50808.60216.90679</t>
-  </si>
-  <si>
-    <t>955.993.998.1001.1006.1009.10424.20103.20125.20310.20384.40151.50623.60159.60162.60192.60225.70103.70113.10425.60126.40139.20205.60280.60274.1048</t>
-  </si>
-  <si>
-    <t>11.20096.20228.20238.20256.20260.20303.20361.40124.50805.60125.60191.60217.60253.61012.90504.90602.90671.90509.20282.60297.1018.60249.1050.60302</t>
-  </si>
-  <si>
-    <t>939.961.962.987.1002.1010.1012.10137.10158.10162.20106.20114.20118.20137.20174.20211.20224.20230.20257.20277.20281.20289.20296.20299.20301.20306.20319.20367.20371.20372.20374.20381.20386.20388.20391.20395.50224.50812.50813.50824.50827.60128.60130.60133.60148.60163.60196.60198.60222.60257.90621.40144.20396.60204.50833.60292.61001.60194.60201</t>
-  </si>
-  <si>
-    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990</t>
-  </si>
-  <si>
-    <t>12.20.265.938.947.970.999.1000.20094.20095.20108.20117.20140.20142.20156.20160.20169.20179.20242.20244.20249.20294.20344.20362.20364.20366.70106.60109.20189.90622.60286.60284.60281.60170.60241.60250.60282.60242.90631.60266.60283.20397.1035.1031.50611.10166.60290.60289.60291.60287.00989.1034.50832.60285.50831.951.1038.1037.50445.1023.1030.1033.1036.1029.50630.1024.1020.1027.1025.1028.50830.1021.1026.1032.20183.1036.1039.1040.60295.1045.60245.60296.1044.921.60243.1.1046.1049.60246.50625.60303.933.50629</t>
+    <t>33.237.251.308.946.950.952.958.963.965.969.10165.20101.20110.20128.20148.20164.20236.20241.20246.20271.20284.20293.20309.20351.20380.20163.50815.50808.60216.90679.20399</t>
+  </si>
+  <si>
+    <t>955.993.998.1001.1006.1009.10424.20103.20125.20310.20384.40151.50623.60159.60162.60192.60225.70103.70113.10425.60126.40139.20205.60280.60274.1048.60288</t>
+  </si>
+  <si>
+    <t>939.961.962.987.1002.1010.1012.10137.10158.10162.20106.20114.20118.20137.20174.20211.20224.20230.20257.20277.20281.20289.20296.20299.20301.20306.20319.20367.20371.20372.20374.20381.20386.20388.20391.20395.50224.50812.50813.50824.50827.60128.60130.60133.60148.60163.60196.60198.60222.60257.90621.40144.20396.60204.50833.60292.61001.60194.60201.1017.60248.1014</t>
+  </si>
+  <si>
+    <t>11.20096.20228.20238.20256.20260.20303.20361.40124.50805.60125.60191.60217.60253.61012.90504.90602.90671.90509.20282.60297.1018.60249.1050.60302.60260.60300.90714.1016.60301</t>
+  </si>
+  <si>
+    <t>936.940.973.992.997.10163.20113.20159.20166.20173.20180.20200.20258.20272.20275.20290.20291.20331.40137.40143.50444.50607.50622.50819.50821.50825.60165.60190.60195.60202.60205.60206.60215.61004.70102.70638.90668.20340.971</t>
+  </si>
+  <si>
+    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943</t>
+  </si>
+  <si>
+    <t>12.20.265.938.947.970.999.1000.20094.20095.20108.20117.20140.20142.20156.20160.20169.20179.20242.20244.20249.20294.20344.20362.20364.20366.70106.60109.20189.90622.60286.60284.60281.60170.60241.60250.60282.60242.90631.60266.60283.20397.1035.1031.50611.10166.60290.60289.60291.60287.00989.1034.50832.60285.50831.951.1038.1037.50445.1023.1030.1033.1036.1029.50630.1024.1020.1027.1025.1028.50830.1021.1026.1032.20183.1036.1039.1040.60295.1045.60245.60296.1044.921.60243.1.1046.1049.60246.50625.60303.933.50629.61007.40146.60240.1041.50610.20306.90630.1047.20398</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -141,16 +127,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -389,7 +373,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -397,7 +381,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -405,7 +389,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -428,8 +412,8 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>17</v>
+      <c r="B7" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -437,7 +421,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -445,14 +429,14 @@
         <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Datos: actualizacion de finanzas y productos; usuarios de oficina 1987 y 1988
</commit_message>
<xml_diff>
--- a/excel/GRUPOS_CLIENTES.xlsx
+++ b/excel/GRUPOS_CLIENTES.xlsx
@@ -57,9 +57,6 @@
     <t>233.10167.20234.20292.20357.20379.20385.50102.50818.60124.60139.60158.60174.60258.70101.3.70114.20129</t>
   </si>
   <si>
-    <t>949.1218.1959.5625.1817.5737</t>
-  </si>
-  <si>
     <t>33.237.251.308.946.950.952.958.963.965.969.10165.20101.20110.20128.20148.20164.20236.20241.20246.20271.20284.20293.20309.20351.20380.20163.50815.50808.60216.90679.20399</t>
   </si>
   <si>
@@ -79,6 +76,9 @@
   </si>
   <si>
     <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943.60247</t>
+  </si>
+  <si>
+    <t>949.1218.1959.5625.1817.5737.1987.1988</t>
   </si>
 </sst>
 </file>
@@ -397,7 +397,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -405,7 +405,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -413,7 +413,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -421,7 +421,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -429,7 +429,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -437,7 +437,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -445,7 +445,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -453,7 +453,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update listas de precios, estado de cuentas
</commit_message>
<xml_diff>
--- a/excel/GRUPOS_CLIENTES.xlsx
+++ b/excel/GRUPOS_CLIENTES.xlsx
@@ -75,10 +75,10 @@
     <t>955.993.998.1001.1006.1009.10424.20103.20125.20310.20384.40151.50623.60159.60162.60192.60225.70103.70113.10425.60126.40139.20205.60280.60274.1048.60288.1051</t>
   </si>
   <si>
-    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943.60247</t>
-  </si>
-  <si>
     <t>949.1218.1959.5625.1817.5737.1987.1988</t>
+  </si>
+  <si>
+    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943.60247.10168</t>
   </si>
 </sst>
 </file>
@@ -405,7 +405,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -421,7 +421,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Datos del dia y cliente de prueba
</commit_message>
<xml_diff>
--- a/excel/GRUPOS_CLIENTES.xlsx
+++ b/excel/GRUPOS_CLIENTES.xlsx
@@ -75,16 +75,16 @@
     <t>936.940.973.992.997.10163.20113.20159.20166.20173.20180.20200.20258.20272.20275.20290.20291.20331.40137.40143.50444.50607.50622.50819.50821.50825.60165.60190.60195.60202.60205.60206.60215.61004.70102.70638.90668.20340.971.20192.60172</t>
   </si>
   <si>
-    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943.60247.10168.20307</t>
-  </si>
-  <si>
     <t>12.20.265.938.947.970.999.1000.20094.20095.20108.20117.20140.20142.20156.20160.20169.20179.20242.20244.20249.20294.20344.20362.20364.20366.70106.60109.20189.90622.60286.60284.60281.60170.60241.60250.60282.60242.90631.60266.60283.20397.1035.1031.50611.10166.60290.60289.60291.60287.00989.1034.50832.60285.50831.951.1038.1037.50445.1023.1030.1033.1036.1029.50630.1024.1020.1027.1025.1028.50830.1021.1026.1032.20183.1036.1039.1040.60295.1045.60245.60296.1044.921.60243.1.1046.1049.60246.50625.60303.933.50629.61007.40146.60240.1041.50610.20306.90630.1047.20398.60306.70117.70118.50226.4.50206</t>
+  </si>
+  <si>
+    <t>5.27.246.920.951.954.956.972.974.980.982.989.994.1005.1007.10107.10157.10160.20109.20116.20120.20121.20146.20165.20178.20201.60270.60134.40125.70115.60150.50230.60278.60299.20267.90713.40147.20337.990.1043.20191.60244.943.60247.10168.20307.7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -421,7 +421,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -429,7 +429,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>